<commit_message>
Refaktor analiz statystycznych OME: powrót do podejścia eksploracyjnego
- Usunięcie poprawki Holma dla wielokrotnych testów w kodzie R (ocena istotności na podstawie surowego p-value).
</commit_message>
<xml_diff>
--- a/PNUW_lato_2025_informacja_OME_to_R.xlsx
+++ b/PNUW_lato_2025_informacja_OME_to_R.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uam-my.sharepoint.com/personal/kp_amu_edu_pl/Documents/nauka/2025_PNUW/PNUW_informacja_OME_2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="986" documentId="8_{037AFBCB-FC45-483C-AFD2-078DE2830EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F273A04B-1768-4782-B5BF-16A2220924B4}"/>
+  <xr:revisionPtr revIDLastSave="989" documentId="8_{037AFBCB-FC45-483C-AFD2-078DE2830EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{523251A0-D770-4A35-B85D-514F64AE484F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="short_colname_data" sheetId="1" r:id="rId1"/>

</xml_diff>